<commit_message>
Add DC stock for SKU-PMP-7700 to fix comprehensive PO test
The new DC-level inventory validator introduced in PR #5 sources from
DC_Stock rows rather than global ATP. The pump SKU had no DC stock
entry, causing the comprehensive happy-path sample to fail with
INVENTORY_SHORTAGE. Added 8 EA at DC-CHI-01 and regenerated all
master data workbooks. All 27/27 tests now pass.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/mock-data/inventory-master-data.xlsx
+++ b/mock-data/inventory-master-data.xlsx
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -894,7 +894,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>DC-DET-02</t>
+          <t>DC-CHI-01</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -909,15 +909,15 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>SKU-STL-4520</t>
+          <t>SKU-PMP-7700</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1200</v>
+        <v>8</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>EA</t>
         </is>
       </c>
     </row>
@@ -939,43 +939,73 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>SKU-VLV-2201</t>
+          <t>SKU-STL-4520</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>15</v>
+        <v>1200</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>FT</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>DC-DET-02</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>DC-LA-05</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>DC</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>SKU-STL-4520</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E10" s="4" t="n">
         <v>2000</v>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>FT</t>
         </is>

</xml_diff>

<commit_message>
Add DC stock for SKU-PMP-7700 to fix comprehensive PO test (#7)
The new DC-level inventory validator introduced in PR #5 sources from
DC_Stock rows rather than global ATP. The pump SKU had no DC stock
entry, causing the comprehensive happy-path sample to fail with
INVENTORY_SHORTAGE. Added 8 EA at DC-CHI-01 and regenerated all
master data workbooks. All 27/27 tests now pass.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/mock-data/inventory-master-data.xlsx
+++ b/mock-data/inventory-master-data.xlsx
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -894,7 +894,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>DC-DET-02</t>
+          <t>DC-CHI-01</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -909,15 +909,15 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>SKU-STL-4520</t>
+          <t>SKU-PMP-7700</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1200</v>
+        <v>8</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>EA</t>
         </is>
       </c>
     </row>
@@ -939,43 +939,73 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>SKU-VLV-2201</t>
+          <t>SKU-STL-4520</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>15</v>
+        <v>1200</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>FT</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>DC-DET-02</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>SKU-VLV-2201</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>DC-LA-05</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>DC</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>West</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>SKU-STL-4520</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E10" s="4" t="n">
         <v>2000</v>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>FT</t>
         </is>

</xml_diff>